<commit_message>
Examens blancs : HG et EMC séparés d'après les relevés officiels, projection expliquée
- Brevet : HG 1,5 + EMC 0,5 ; 1re et Terminale : HG 3 + EMC 1 (totaux inchangés)
- Modèle d'import : colonnes HG et EMC séparées (ancienne colonne commune acceptée)
- Base : code EMC pour les notes officielles ; T53 ajusté
- Projection au bac : explication pas à pas à l'écran

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015H2hcPvamfd6F2wHY6EoXt
</commit_message>
<xml_diff>
--- a/ent/modeles/modele-import-chateaubriand.xlsx
+++ b/ent/modeles/modele-import-chateaubriand.xlsx
@@ -1692,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1702,9 +1702,10 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1740,20 +1741,25 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Histoire-géo et EMC</t>
+          <t>Histoire-géographie</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>EMC</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>Ens. scientifique (ou maths STMG)</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>LVA</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>LVB</t>
         </is>
@@ -1797,15 +1803,20 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>12</t>
         </is>

</xml_diff>

<commit_message>
Import de l'emploi du temps (format de l'école, semaines A/B) et écran Emplois du temps
- Lecture du fichier « EDT à importer » ou de l'onglet 4 du modèle : abréviations de classes et de
  matières, enseignement scientifique partagé, semaines A/B, contrôles et chevauchements
- Compte rendu avant import, heures par classe ; agenda et changements d'emploi du temps branchés
- Écran Emplois du temps par classe ou par professeur, semaine A ou B, imprimable
- Modèle Excel : onglet 4 au format de l'école

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015H2hcPvamfd6F2wHY6EoXt
</commit_message>
<xml_diff>
--- a/ent/modeles/modele-import-chateaubriand.xlsx
+++ b/ent/modeles/modele-import-chateaubriand.xlsx
@@ -264,12 +264,22 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>HH:MM</t>
+        <t>HH:MM-HH:MM</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>HH:MM</t>
+        <t>Abréviations comprises : HGE, P-C, Spé Maths, E.S. SVT…</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Facultatif</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>A, B ou vide</t>
       </text>
     </comment>
   </commentList>
@@ -765,7 +775,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4 Emploi du temps — Une ligne par cours de la semaine type.</t>
+          <t>4 Emploi du temps — Une ligne par cours de la semaine type. Semaine : A ou B pour un cours une semaine sur deux, vide sinon.</t>
         </is>
       </c>
     </row>
@@ -1464,49 +1474,49 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>Jour</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Jour</t>
-        </is>
-      </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Début</t>
+          <t>Créneau horaire</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Matière</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Matière</t>
+          <t>Enseignant</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Professeur</t>
+          <t>Salle</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Salle</t>
+          <t>Semaine</t>
         </is>
       </c>
     </row>
@@ -1518,42 +1528,38 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>1re STMG</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>07:30-09:30</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>Management</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Mme Exemple</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Mme Exemple</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
           <t>Salle 12</t>
         </is>
       </c>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="A2:A2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisissez une valeur dans la liste." type="list">
-      <formula1>"6e,5e,4e,3e,2de,1re Générale,1re STMG,Terminale Générale,Terminale STMG"</formula1>
+      <formula1>"Lundi,Mardi,Mercredi,Jeudi,Vendredi,Samedi"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisissez une valeur dans la liste." type="list">
-      <formula1>"Lundi,Mardi,Mercredi,Jeudi,Vendredi,Samedi"</formula1>
+      <formula1>"6e,5e,4e,3e,2de,1re Générale,1re STMG,Terminale Générale,Terminale STMG"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>